<commit_message>
chore(data): rebuild team KPIs and team master table with real-PIR funnel
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/curated/team_kpis.xlsx
+++ b/data/curated/team_kpis.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Team KPIs" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Guide'!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Team KPIs'!$A$1:$G$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Guide'!$A$1:$C$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Team KPIs'!$A$1:$J$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,11 +429,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -573,8 +573,59 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Team KPIs</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>funnel_actual_pir_guards</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Real-PIR analogue of funnel_ratio_guards: PIR (Kaggle box score) of the opposing guards who played, summed per game and averaged over the team's games, / the 20-team league average; 1.0 = league-average PIR conceded to guards, &gt;1 = concedes more than average. Position from the player master table (G/F/C); postseason games included</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Team KPIs</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>funnel_actual_pir_forwards</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Real-PIR analogue of funnel_ratio_forwards: PIR of the opposing forwards who played, summed per game and averaged over the team's games, / the 20-team league average for forwards</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Team KPIs</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>funnel_actual_pir_centers</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Real-PIR analogue of funnel_ratio_centers: PIR of the opposing centers who played, summed per game and averaged over the team's games, / the 20-team league average for centers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C8"/>
+  <autoFilter ref="A1:C11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -585,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -595,6 +646,9 @@
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -633,6 +687,21 @@
           <t>funnel_ratio_centers</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>funnel_actual_pir_guards</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>funnel_actual_pir_forwards</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>funnel_actual_pir_centers</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -658,6 +727,15 @@
       <c r="G2" t="n">
         <v>1.018886846063848</v>
       </c>
+      <c r="H2" t="n">
+        <v>0.9390987132899038</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1.086306244359849</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.9881512371268025</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -683,6 +761,15 @@
       <c r="G3" t="n">
         <v>1.010195554069865</v>
       </c>
+      <c r="H3" t="n">
+        <v>0.9487130980791247</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.9802915228378812</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1.052076896816481</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -708,6 +795,15 @@
       <c r="G4" t="n">
         <v>0.9600534848738091</v>
       </c>
+      <c r="H4" t="n">
+        <v>1.000822783041774</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.002858225588581</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.9196385090610945</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -733,6 +829,15 @@
       <c r="G5" t="n">
         <v>0.9660705331773357</v>
       </c>
+      <c r="H5" t="n">
+        <v>1.033882477480223</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1.007760226691265</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.986674179971157</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -758,6 +863,15 @@
       <c r="G6" t="n">
         <v>0.9901387263914425</v>
       </c>
+      <c r="H6" t="n">
+        <v>1.097071653607103</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.9440342123563761</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.9467936367687301</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -783,6 +897,15 @@
       <c r="G7" t="n">
         <v>1.01754972421862</v>
       </c>
+      <c r="H7" t="n">
+        <v>0.9400398286790275</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.9207668071224749</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1.100112169524727</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -808,6 +931,15 @@
       <c r="G8" t="n">
         <v>0.9921444091592847</v>
       </c>
+      <c r="H8" t="n">
+        <v>0.9572487957944331</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.080378243026371</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1.023600608862293</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -833,6 +965,15 @@
       <c r="G9" t="n">
         <v>0.9908072873140565</v>
       </c>
+      <c r="H9" t="n">
+        <v>0.8809903096126125</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.8977820159056348</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.999864643872735</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -858,6 +999,15 @@
       <c r="G10" t="n">
         <v>0.8443924452615745</v>
       </c>
+      <c r="H10" t="n">
+        <v>0.9469733522601228</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1.036482804580855</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.8967143655868465</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -883,6 +1033,15 @@
       <c r="G11" t="n">
         <v>1.046297843891025</v>
       </c>
+      <c r="H11" t="n">
+        <v>1.101777230552722</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1.115946251027239</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.9453165796130846</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -908,6 +1067,15 @@
       <c r="G12" t="n">
         <v>1.18335283302691</v>
       </c>
+      <c r="H12" t="n">
+        <v>1.11858286250136</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1.010724227358004</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1.116655209667956</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -933,6 +1101,15 @@
       <c r="G13" t="n">
         <v>1.079725890021728</v>
       </c>
+      <c r="H13" t="n">
+        <v>1.084299373326138</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1.057407237859143</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1.184599838827647</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -958,6 +1135,15 @@
       <c r="G14" t="n">
         <v>0.8229984957379242</v>
       </c>
+      <c r="H14" t="n">
+        <v>0.9891091473398514</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.8460498647338294</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.7740466498910338</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -983,6 +1169,15 @@
       <c r="G15" t="n">
         <v>0.8089587163630286</v>
       </c>
+      <c r="H15" t="n">
+        <v>1.08506326568744</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.9560923059778825</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.8699866646751669</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1008,6 +1203,15 @@
       <c r="G16" t="n">
         <v>1.274945679425038</v>
       </c>
+      <c r="H16" t="n">
+        <v>1.075560444712846</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1.040364234025394</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1.249590353676046</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1033,6 +1237,15 @@
       <c r="G17" t="n">
         <v>1.217449440080227</v>
       </c>
+      <c r="H17" t="n">
+        <v>0.9780877794107445</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1.099644247360174</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1.138811067002638</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1058,6 +1271,15 @@
       <c r="G18" t="n">
         <v>0.7621594517800435</v>
       </c>
+      <c r="H18" t="n">
+        <v>0.9619849284345038</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.8524196462935338</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.7896213276157307</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1083,6 +1305,15 @@
       <c r="G19" t="n">
         <v>0.9292996824335618</v>
       </c>
+      <c r="H19" t="n">
+        <v>0.9567599046831999</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1.082163379791566</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.848300780071827</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1108,6 +1339,15 @@
       <c r="G20" t="n">
         <v>1.071703158950359</v>
       </c>
+      <c r="H20" t="n">
+        <v>1.011699043308021</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1.014429228191428</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1.141765181313929</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1133,9 +1373,18 @@
       <c r="G21" t="n">
         <v>1.012869797760321</v>
       </c>
+      <c r="H21" t="n">
+        <v>0.8922350081988442</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.968099074912519</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1.027680100054076</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G21"/>
+  <autoFilter ref="A1:J21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>